<commit_message>
Update 8 subclusters (factoriescap_s (usage) 0 visnorm).xlsx
</commit_message>
<xml_diff>
--- a/clustering/8 subclusters (factoriescap_s (usage) 0 visnorm).xlsx
+++ b/clustering/8 subclusters (factoriescap_s (usage) 0 visnorm).xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="14">
   <si>
     <t>clust</t>
   </si>
@@ -84,6 +84,8 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <sz val="11"/>
@@ -227,7 +229,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -296,6 +298,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -651,7 +656,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.28515625" customWidth="1"/>
@@ -1064,8 +1069,197 @@
         <v>21.99999999999979</v>
       </c>
     </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <v>0</v>
+      </c>
+      <c r="B31" s="2">
+        <v>239537.8512039996</v>
+      </c>
+      <c r="C31" s="2">
+        <v>1418</v>
+      </c>
+      <c r="D31" s="24">
+        <f>D24/$C24</f>
+        <v>4.3981481481481455E-2</v>
+      </c>
+      <c r="E31" s="24">
+        <f>E24/$C24</f>
+        <v>0.22222222222222246</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <v>1</v>
+      </c>
+      <c r="B32" s="2">
+        <v>1615284.14922</v>
+      </c>
+      <c r="C32" s="2">
+        <v>5560.5</v>
+      </c>
+      <c r="D32" s="24">
+        <f t="shared" ref="D32:E34" si="1">D25/$C25</f>
+        <v>4.290718038528895E-2</v>
+      </c>
+      <c r="E32" s="24">
+        <f t="shared" si="1"/>
+        <v>0.20753064798598922</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>2</v>
+      </c>
+      <c r="B33" s="2">
+        <v>1418484.1690199999</v>
+      </c>
+      <c r="C33" s="2">
+        <v>4248.5</v>
+      </c>
+      <c r="D33" s="24">
+        <f t="shared" si="1"/>
+        <v>4.6473482777474026E-2</v>
+      </c>
+      <c r="E33" s="24">
+        <f t="shared" si="1"/>
+        <v>0.19445963185711665</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <v>3</v>
+      </c>
+      <c r="B34" s="2">
+        <v>578868.78119999985</v>
+      </c>
+      <c r="C34" s="2">
+        <v>2406.9999999999991</v>
+      </c>
+      <c r="D34" s="24">
+        <f t="shared" si="1"/>
+        <v>3.2258064516129274E-2</v>
+      </c>
+      <c r="E34" s="24">
+        <f t="shared" si="1"/>
+        <v>0.17741935483871013</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B9">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C9">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D9">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E9">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B24:B27">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C24:C27">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D24:D27">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E24:E27">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B31:B34">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -1077,7 +1271,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C9">
+  <conditionalFormatting sqref="C31:C34">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -1089,7 +1283,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D9">
+  <conditionalFormatting sqref="D31:D34">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1101,7 +1295,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E9">
+  <conditionalFormatting sqref="E31:E34">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>